<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table35-39
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table36.xlsx
+++ b/sources/table_normalization/xlsx/economy-table36.xlsx
@@ -179,8 +179,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -327,7 +327,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -341,52 +341,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -396,20 +372,47 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -686,113 +689,117 @@
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" customWidth="1"/>
+    <col min="1" max="1" width="20.26953125" customWidth="1"/>
     <col min="4" max="4" width="12.54296875" customWidth="1"/>
     <col min="5" max="5" width="11.90625" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="11.453125" customWidth="1"/>
     <col min="10" max="10" width="13.36328125" customWidth="1"/>
     <col min="11" max="11" width="14.453125" customWidth="1"/>
     <col min="12" max="12" width="14.08984375" customWidth="1"/>
     <col min="13" max="13" width="14.1796875" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="10.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="12" t="s">
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="12"/>
-      <c r="L1" s="13" t="s">
+      <c r="K1" s="17"/>
+      <c r="L1" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13" t="s">
+      <c r="M1" s="18"/>
+      <c r="N1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="13"/>
+      <c r="O1" s="18"/>
     </row>
     <row r="2" spans="1:15" ht="32.5" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="14" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="23"/>
+      <c r="F2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="15"/>
-      <c r="H2" s="14" t="s">
+      <c r="G2" s="23"/>
+      <c r="H2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="15"/>
-      <c r="J2" s="16" t="s">
+      <c r="I2" s="23"/>
+      <c r="J2" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="N2" s="14" t="s">
+      <c r="M2" s="23"/>
+      <c r="N2" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="15"/>
+      <c r="O2" s="23"/>
     </row>
     <row r="3" spans="1:15" ht="37.5">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="18" t="s">
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="O3" s="27" t="s">
         <v>16</v>
       </c>
     </row>
@@ -813,10 +820,10 @@
       <c r="E4" s="5">
         <v>1.71585365853659</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="12">
         <v>1</v>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="13">
         <v>0</v>
       </c>
       <c r="H4" s="6">
@@ -865,10 +872,10 @@
       <c r="E5" s="5">
         <v>1.6700975609756099</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="12">
         <v>12</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="13">
         <v>0</v>
       </c>
       <c r="H5" s="6">
@@ -917,10 +924,10 @@
       <c r="E6" s="5">
         <v>1.4094512195122</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="12">
         <v>10</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="13">
         <v>0</v>
       </c>
       <c r="H6" s="6">
@@ -969,10 +976,10 @@
       <c r="E7" s="5">
         <v>1.3481707317073199</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="12">
         <v>20</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="13">
         <v>6</v>
       </c>
       <c r="H7" s="6">
@@ -1021,10 +1028,10 @@
       <c r="E8" s="5">
         <v>1.26646341463415</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="12">
         <v>10</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="13">
         <v>6</v>
       </c>
       <c r="H8" s="6">

</xml_diff>